<commit_message>
fix(ep-testing): cart-order and payment-payos
</commit_message>
<xml_diff>
--- a/docs/testing/EP/payment_payos/Testcase_EP_Payment_PayOS.xlsx
+++ b/docs/testing/EP/payment_payos/Testcase_EP_Payment_PayOS.xlsx
@@ -997,7 +997,7 @@
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Không cập nhật PAID, ghi nhận hủy thanh toán (HTTP 200)</t>
+          <t>Không cập nhật PAID, giữ nguyên UNPAID (HTTP 200)</t>
         </is>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1104,7 +1104,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Thanh toán đơn hàng đơn lẻ bằng tiền mặt (CASH) thành công khi đơn READY</t>
+          <t>Thanh toán đơn hàng bằng tiền mặt (CASH) thành công khi đơn READY</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>HTTP 200 OK. Thanh toán thành công, mở bàn ăn.</t>
+          <t>HTTP 200 OK. Xác nhận thanh toán thành công.</t>
         </is>
       </c>
       <c r="L2" s="7" t="inlineStr">
@@ -1171,12 +1171,12 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Tạo link thanh toán PayOS thành công cho đơn hàng</t>
+          <t>Tạo link thanh toán PayOS thành công cho đơn hàng hợp lệ</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>EQ_AMT1, EQ_MTH1 (Valid)</t>
+          <t>EQ_AMT1 (Valid)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -1196,13 +1196,13 @@
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>1. Gửi POST /api/payos/create-payment-link với orderId = 1
+          <t>1. Gửi POST /api/payos/create-payment-link với orderId: {{order_id}}
 2. Kiểm tra checkoutUrl trả về</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>Body: {"orderId": 1}</t>
+          <t>Body: {"orderId": {{order_id}}}</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -1235,7 +1235,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Xử lý Webhook PayOS khi khách hàng thanh toán thành công (code = '00')</t>
+          <t>Xử lý Webhook PayOS khi thanh toán thành công (code = '00'), kiểm tra đơn chuyển PAID &amp; COMPLETED</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -1261,7 +1261,8 @@
       <c r="H4" s="4" t="inlineStr">
         <is>
           <t>1. Gửi POST /api/payos/webhook với code = '00'
-2. Kiểm tra cập nhật đơn hàng</t>
+2. Kiểm tra phản hồi Webhook 200
+3. Gửi GET kiểm tra trạng thái đơn</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
@@ -1273,12 +1274,12 @@
       <c r="J4" s="4" t="inlineStr">
         <is>
           <t>Status: 200 OK
-message: 'Success', đơn chuyển PAID/COMPLETED, bàn chuyển AVAILABLE.</t>
+message: 'Success', đơn hàng thực tế chuyển sang PAID và COMPLETED.</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>HTTP 200 OK. Xử lý Webhook thành công 200.</t>
+          <t>HTTP 200 OK. Webhook thành công &amp; đơn hàng chuyển PAID/COMPLETED.</t>
         </is>
       </c>
       <c r="L4" s="7" t="inlineStr">
@@ -1343,7 +1344,7 @@
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>HTTP 400 Bad Request. Chặn thanh toán đơn chưa hoàn thành.</t>
+          <t>HTTP 400 Bad Request. Báo lỗi trạng thái đơn không hợp lệ.</t>
         </is>
       </c>
       <c r="L5" s="7" t="inlineStr">
@@ -1408,7 +1409,7 @@
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>HTTP 400 Bad Request. Từ chối thanh toán trùng lặp.</t>
+          <t>HTTP 400 Bad Request. Báo lỗi đơn đã được thanh toán trước đó.</t>
         </is>
       </c>
       <c r="L6" s="7" t="inlineStr">
@@ -1430,7 +1431,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Xử lý Webhook PayOS khi giao dịch bị hủy (code = '01')</t>
+          <t>Xử lý Webhook PayOS khi giao dịch bị hủy (code = '01'), kiểm tra đơn giữ UNPAID</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -1456,7 +1457,8 @@
       <c r="H7" s="4" t="inlineStr">
         <is>
           <t>1. Gửi POST /api/payos/webhook với code = '01'
-2. Kiểm tra trạng thái đơn</t>
+2. Kiểm tra phản hồi 200
+3. Gửi GET kiểm tra đơn giữ UNPAID</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -1467,15 +1469,207 @@
       <c r="J7" s="4" t="inlineStr">
         <is>
           <t>Status: 200 OK
-Ghi nhận giao dịch không thành công, không cập nhật đơn sang PAID.</t>
+message: 'Success', đơn hàng không bị chuyển sang PAID (vẫn UNPAID).</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>HTTP 200 OK. Ghi nhận hủy giao dịch an toàn.</t>
+          <t>HTTP 200 OK. Ghi nhận hủy an toàn và đơn giữ UNPAID.</t>
         </is>
       </c>
       <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>TC_EP_PAY_07</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>PayOS</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Từ chối tạo link thanh toán khi số tiền dưới mức tối thiểu (amount &lt; 1.000 VNĐ)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>EQ_AMT2 (Invalid)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>/api/payos/create-payment-link</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Có auth token hợp lệ</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>1. Gửi POST /api/payos/create-payment-link với amount = 500
+2. Kiểm tra bắt lỗi hạn mức</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>Body: {"orderId": 99999999, "amount": 500}</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>Status: 400 Bad Request
+Báo lỗi số tiền dưới mức tối thiểu 1.000 VNĐ.</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 400 Bad Request. Chặn giao dịch dưới hạn mức tối thiểu.</t>
+        </is>
+      </c>
+      <c r="L8" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>TC_EP_PAY_08</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>PayOS</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Từ chối tạo link thanh toán khi số tiền vượt hạn mức tối đa (amount &gt; 500.000.000 VNĐ)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>EQ_AMT3 (Invalid)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>/api/payos/create-payment-link</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Có auth token hợp lệ</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>1. Gửi POST /api/payos/create-payment-link với amount = 600.000.000
+2. Kiểm tra bắt lỗi hạn mức</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>Body: {"orderId": 99999999, "amount": 600000000}</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>Status: 400 Bad Request
+Báo lỗi số tiền vượt quá hạn mức tối đa 500.000.000 VNĐ.</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 400 Bad Request. Chặn giao dịch vượt hạn mức tối đa.</t>
+        </is>
+      </c>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>TC_EP_PAY_09</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Payment</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Từ chối thanh toán khi phương thức thanh toán không được hỗ trợ (paymentMethod = 'BITCOIN')</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>EQ_MTH2 (Invalid)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>/api/orders/{{order_id}}/pay</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Có auth token hợp lệ</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>1. Gửi PUT thanh toán đơn với phương thức BITCOIN
+2. Kiểm tra bắt lỗi phương thức</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>Body: {"paymentMethod": "BITCOIN"}</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>Status: 400 Bad Request
+Báo lỗi phương thức thanh toán không hỗ trợ.</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>HTTP 400 Bad Request. Từ chối phương thức thanh toán không hợp lệ.</t>
+        </is>
+      </c>
+      <c r="L10" s="7" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>

</xml_diff>